<commit_message>
developed employee module with some pending components to complete
</commit_message>
<xml_diff>
--- a/EMS Timeline.xlsx
+++ b/EMS Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookair/Documents/Work/Developments/Apptron Solutions/2026-06-15 Employee Management System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F461476-3F41-4A4C-8CC0-692CBD3B1947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6F6984-D3BC-7841-B712-CFA93DA1BD50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="480" windowWidth="28800" windowHeight="17520" xr2:uid="{ACEAC283-D276-4040-BACC-DCABDF7C78AB}"/>
   </bookViews>
@@ -407,27 +407,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -455,16 +435,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1091,7 +1061,7 @@
         <v>26</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -1102,7 +1072,7 @@
         <v>28</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
@@ -1120,7 +1090,7 @@
         <v>29</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
@@ -1131,7 +1101,7 @@
         <v>30</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
@@ -1685,13 +1655,13 @@
     <mergeCell ref="A47:C47"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="pending">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="in progress">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="in progress">
       <formula>NOT(ISERROR(SEARCH("in progress",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",C1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Implement JWT authentication backend
</commit_message>
<xml_diff>
--- a/EMS Timeline.xlsx
+++ b/EMS Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookair/Documents/Work/Developments/Apptron Solutions/2026-06-15 Employee Management System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6F6984-D3BC-7841-B712-CFA93DA1BD50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0649D3BB-158A-E24E-987C-DC9DBBEA9B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="480" windowWidth="28800" windowHeight="17520" xr2:uid="{ACEAC283-D276-4040-BACC-DCABDF7C78AB}"/>
   </bookViews>
@@ -177,9 +177,6 @@
     <t>Password Hashing</t>
   </si>
   <si>
-    <t>Login/Register/Logout APIs</t>
-  </si>
-  <si>
     <t>Middleware</t>
   </si>
   <si>
@@ -298,6 +295,9 @@
   </si>
   <si>
     <t>completed</t>
+  </si>
+  <si>
+    <t>Login/Logout APIs</t>
   </si>
 </sst>
 </file>
@@ -394,13 +394,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -420,21 +420,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -751,518 +751,518 @@
   <dimension ref="A1:C84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.5" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.5" style="3" customWidth="1"/>
     <col min="3" max="3" width="14.5" style="2" customWidth="1"/>
     <col min="4" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
+      <c r="A2" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="6">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="6">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="6">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="6">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="6">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="6">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="6">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="6">
+      <c r="A10" s="4">
         <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="6">
+      <c r="A11" s="4">
         <v>9</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="6">
+      <c r="A12" s="4">
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="6">
+      <c r="A13" s="4">
         <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="6">
+      <c r="A14" s="4">
         <v>12</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="6">
+      <c r="A15" s="4">
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="6">
+      <c r="A16" s="4">
         <v>14</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
+      <c r="A17" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="6">
+      <c r="A18" s="4">
         <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" s="6">
+      <c r="A19" s="4">
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" s="6">
+      <c r="A20" s="4">
         <v>17</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="6">
+      <c r="A21" s="4">
         <v>18</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="6">
+      <c r="A22" s="4">
         <v>19</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="6">
+      <c r="A23" s="4">
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="6">
+      <c r="A24" s="4">
         <v>21</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="6">
+      <c r="A25" s="4">
         <v>22</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
+      <c r="A26" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="6">
+      <c r="A27" s="4">
         <v>23</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" s="6">
+      <c r="A28" s="4">
         <v>24</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" s="6">
+      <c r="A29" s="4">
         <v>25</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>26</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="6">
+      <c r="A30" s="4">
         <v>26</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
+      <c r="A31" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" s="6">
+      <c r="A32" s="4">
         <v>27</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="6">
+      <c r="A33" s="4">
         <v>28</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>30</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="6">
+      <c r="A34" s="4">
         <v>29</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>31</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="6">
+      <c r="A35" s="4">
         <v>30</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>32</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="6">
+      <c r="A36" s="4">
         <v>31</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="6">
+      <c r="A37" s="4">
         <v>32</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>34</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
+      <c r="A38" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="6">
+      <c r="A39" s="4">
         <v>33</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>35</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="6">
+      <c r="A40" s="4">
         <v>34</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="6">
+      <c r="A41" s="4">
         <v>35</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>37</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="6">
+      <c r="A42" s="4">
         <v>36</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="6">
+      <c r="A43" s="4">
         <v>37</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>39</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="6">
+      <c r="A44" s="4">
         <v>38</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>40</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="6">
+      <c r="A45" s="4">
         <v>39</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="6">
+      <c r="A46" s="4">
         <v>40</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
+      <c r="A47" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="6">
+      <c r="A48" s="4">
         <v>41</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>42</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="6">
+      <c r="A49" s="4">
         <v>42</v>
       </c>
       <c r="B49" s="3" t="s">
@@ -1273,372 +1273,372 @@
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="6">
+      <c r="A50" s="4">
         <v>43</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="6">
+      <c r="A51" s="4">
         <v>44</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="6">
+      <c r="A52" s="4">
         <v>45</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="6">
+      <c r="A53" s="4">
         <v>46</v>
       </c>
       <c r="B53" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="4">
         <v>47</v>
       </c>
-      <c r="C53" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="6">
+      <c r="B54" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="C54" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B55" s="5"/>
+      <c r="C55" s="5"/>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="4">
         <v>48</v>
       </c>
-      <c r="C54" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="4" t="s">
+      <c r="B56" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="4">
+        <v>49</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="4">
+        <v>50</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="4">
+        <v>51</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="4">
+        <v>52</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="4">
+        <v>53</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B55" s="4"/>
-      <c r="C55" s="4"/>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="6">
-        <v>48</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="6">
-        <v>49</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="6">
-        <v>50</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="6">
-        <v>51</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="6">
-        <v>52</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="6">
-        <v>53</v>
-      </c>
-      <c r="B61" s="3" t="s">
+      <c r="B62" s="5"/>
+      <c r="C62" s="5"/>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="4">
         <v>54</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="4" t="s">
+      <c r="B63" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="4">
+        <v>55</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="4">
+        <v>56</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="4">
+        <v>57</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="4">
+        <v>58</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="4">
+        <v>59</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B62" s="4"/>
-      <c r="C62" s="4"/>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="6">
-        <v>54</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="6">
-        <v>55</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="6">
-        <v>56</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="6">
-        <v>57</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="6">
-        <v>58</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="6">
-        <v>59</v>
-      </c>
-      <c r="B68" s="3" t="s">
+      <c r="B69" s="5"/>
+      <c r="C69" s="5"/>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="4">
         <v>60</v>
       </c>
-      <c r="C68" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="4" t="s">
+      <c r="B70" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="4">
+        <v>61</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="4">
+        <v>62</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="4">
+        <v>63</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="4">
+        <v>64</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="4">
+        <v>65</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B69" s="4"/>
-      <c r="C69" s="4"/>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="6">
-        <v>60</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="6">
-        <v>61</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="6">
-        <v>62</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" s="6">
-        <v>63</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="6">
-        <v>64</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="6">
-        <v>65</v>
-      </c>
-      <c r="B75" s="3" t="s">
+      <c r="B76" s="5"/>
+      <c r="C76" s="5"/>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="4">
         <v>66</v>
       </c>
-      <c r="C75" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="B76" s="4"/>
-      <c r="C76" s="4"/>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="6">
+      <c r="B77" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="C77" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78" s="4">
         <v>67</v>
       </c>
-      <c r="C77" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A78" s="6">
+      <c r="B78" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="C78" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A79" s="4">
         <v>68</v>
       </c>
-      <c r="C78" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A79" s="6">
+      <c r="B79" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="C79" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A80" s="4">
         <v>69</v>
       </c>
-      <c r="C79" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" s="6">
+      <c r="B80" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="C80" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A81" s="4">
         <v>70</v>
       </c>
-      <c r="C80" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" s="6">
+      <c r="B81" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B81" s="3" t="s">
+      <c r="C81" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A82" s="4">
         <v>71</v>
       </c>
-      <c r="C81" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" s="6">
+      <c r="B82" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B82" s="3" t="s">
+      <c r="C82" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83" s="4">
         <v>72</v>
       </c>
-      <c r="C82" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" s="6">
+      <c r="B83" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B83" s="3" t="s">
+      <c r="C83" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A84" s="4">
         <v>73</v>
       </c>
-      <c r="C83" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" s="6">
+      <c r="B84" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B84" s="3" t="s">
-        <v>74</v>
-      </c>
       <c r="C84" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1655,10 +1655,10 @@
     <mergeCell ref="A47:C47"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="pending">
+    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="in progress">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="in progress">
       <formula>NOT(ISERROR(SEARCH("in progress",C1)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="completed">

</xml_diff>

<commit_message>
Add Employee Form completed
</commit_message>
<xml_diff>
--- a/EMS Timeline.xlsx
+++ b/EMS Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookair/Documents/Work/Developments/Apptron Solutions/2026-06-15 Employee Management System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0649D3BB-158A-E24E-987C-DC9DBBEA9B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF57F4E-70BF-8043-9462-E23C4DEF11DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="480" windowWidth="28800" windowHeight="17520" xr2:uid="{ACEAC283-D276-4040-BACC-DCABDF7C78AB}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="89">
   <si>
     <t>#</t>
   </si>
@@ -298,6 +298,9 @@
   </si>
   <si>
     <t>Login/Logout APIs</t>
+  </si>
+  <si>
+    <t>not needed</t>
   </si>
 </sst>
 </file>
@@ -407,7 +410,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="7">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -435,6 +438,46 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2" tint="-0.89996032593768116"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -904,7 +947,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -926,7 +969,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -955,7 +998,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -966,7 +1009,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -977,7 +1020,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -1112,7 +1155,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
@@ -1269,7 +1312,7 @@
         <v>43</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
@@ -1302,7 +1345,7 @@
         <v>46</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
@@ -1313,7 +1356,7 @@
         <v>87</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
@@ -1324,7 +1367,7 @@
         <v>47</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
@@ -1342,7 +1385,7 @@
         <v>48</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
@@ -1353,7 +1396,7 @@
         <v>49</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
@@ -1459,7 +1502,7 @@
         <v>58</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
@@ -1470,7 +1513,7 @@
         <v>59</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -1655,14 +1698,17 @@
     <mergeCell ref="A47:C47"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="pending">
+    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="in progress">
+    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="in progress">
       <formula>NOT(ISERROR(SEARCH("in progress",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",C1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="not needed">
+      <formula>NOT(ISERROR(SEARCH("not needed",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>